<commit_message>
feat: implement MISRA configuration modal and warning viewer with associated UI components and logic
</commit_message>
<xml_diff>
--- a/Output_excel_after_run/audit_report.xlsx
+++ b/Output_excel_after_run/audit_report.xlsx
@@ -548,12 +548,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>uint16_t small;</t>
+          <t>small = (uint8_t)(total + 300);</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>20260402_141558_18f222fa</t>
+          <t>20260402_175445_1770186c</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-04-02 14:22:14</t>
+          <t>2026-04-02 18:04:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement web interface for MISRA compliance reviewer with server-side processing and result visualization
</commit_message>
<xml_diff>
--- a/Output_excel_after_run/audit_report.xlsx
+++ b/Output_excel_after_run/audit_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -553,7 +553,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>20260402_175445_1770186c</t>
+          <t>20260405_161935_e6a0c033</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-04-02 18:04:23</t>
+          <t>2026-04-05 16:25:23</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>20260402_145450_3d4e2eb1</t>
+          <t>20260405_203102_431f6a95</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -644,7 +644,114 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-04-02 15:03:18</t>
+          <t>2026-04-05 20:33:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3673</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>8.13</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Pointer parameter should be const</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>logger.c</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>log_message</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       1  #include &lt;stdio.h&gt;
+       2  #include &lt;string.h&gt;
+       3  
+       4  static char log_buffer[64];
+       5  
+       6  void log_message(char * msg)
+       7  {
+       8      int status = 0;
+       9  
+      10      strcpy(log_buffer, msg);
+      11  
+      12      status = puts(log_buffer);
+      13  
+      14      status = status;
+      15  }</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>6  void log_message(const char * msg)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>20260405_201752_56ba16ef</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-04-05 20:22:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3200</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1  #include &lt;stdio.h&gt;
+       2  #include &lt;string.h&gt;
+       3  
+       4  static char log_buffer[64];
+       5  
+       6  void log_message(char * msg)
+       7  {
+       8      int status = 0;
+       9  
+      10      strcpy(log_buffer, msg);
+      11  
+      12      status = puts(log_buffer);
+      13  
+      14      printf("puts returned: %d\n", status);
+      15  }</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-04-05 19:21:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement web server, orchestration pipeline, and supporting data infrastructure for MISRA analysis
</commit_message>
<xml_diff>
--- a/Output_excel_after_run/audit_report.xlsx
+++ b/Output_excel_after_run/audit_report.xlsx
@@ -51,7 +51,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -88,11 +88,6 @@
         <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF9C4"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -106,10 +101,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -117,11 +115,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -135,20 +130,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -515,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -530,9 +516,10 @@
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="55" customWidth="1" min="11" max="11"/>
     <col width="55" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -573,40 +560,45 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Fix 2</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Chosen Fix</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Chosen Fix Code</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Violated Source Code</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Fixed Code (Full File)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>User Edited &amp; Committed</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Audit Status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Run ID</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
@@ -641,47 +633,52 @@
           <t>main</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H2" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I2" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J2" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K2" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L2" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M2" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N2" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O2" s="12" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -716,47 +713,52 @@
           <t>main</t>
         </is>
       </c>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K3" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L3" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M3" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N3" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O3" s="12" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -791,47 +793,52 @@
           <t>helper_add</t>
         </is>
       </c>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H4" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K4" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L4" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M4" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N4" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O4" s="12" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -866,47 +873,52 @@
           <t>update_index</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K5" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L5" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M5" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N5" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O5" s="12" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -941,47 +953,52 @@
           <t>early_return</t>
         </is>
       </c>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H6" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I6" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K6" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L6" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M6" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N6" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O6" s="12" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1016,53 +1033,58 @@
           <t>factorial</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H7" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I7" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J7" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K7" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L7" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M7" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N7" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O7" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="100" customHeight="1">
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" t="n">
         <v>2883</v>
       </c>
@@ -1093,80 +1115,52 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>[Initialize 'raw_value' before reading it]
-5      int raw_value = 0;</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>User Edited</t>
-        </is>
-      </c>
-      <c r="I8" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>#include &lt;stdint.h&gt;
-int read_sensor(void)
-{
-    int raw_value = 0;
-    int output = 0;
-    if (output == 0)
-    {
-        output = raw_value;
-    }
-    return output;
-}
-uint8_t scale_value(uint16_t input)
-{
-    uint8_t scaled;
-    scaled = input;
-    return scaled;
-}</t>
-        </is>
-      </c>
-      <c r="L8" s="7" t="inlineStr">
-        <is>
-          <t>#include &lt;stdint.h&gt;
-int read_sensor(void)
-{
-    int raw_value = 0;
-    int output = 0;
-    if (output == 0)
-    {
-        output = raw_value;
-    }
-    return output;
-}
-uint8_t scale_value(uint16_t input)
-{
-    uint8_t scaled;
-    scaled = input;
-    return scaled;
-}</t>
-        </is>
-      </c>
-      <c r="M8" s="8" t="inlineStr">
-        <is>
-          <t>User Edited &amp; Committed</t>
-        </is>
-      </c>
-      <c r="N8" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O8" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-07 17:25:23</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1199,47 +1193,52 @@
           <t>scale_value</t>
         </is>
       </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H9" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I9" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K9" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L9" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M9" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N9" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O9" s="12" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1274,47 +1273,52 @@
           <t>log_message</t>
         </is>
       </c>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H10" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I10" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L10" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M10" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N10" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O10" s="12" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1349,47 +1353,52 @@
           <t>log_message</t>
         </is>
       </c>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H11" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I11" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K11" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L11" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M11" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N11" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O11" s="12" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1404,9 +1413,9 @@
           <t>MISRA-R (Required)</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>14.4</t>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Rule 14.4</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1424,36 +1433,35 @@
           <t>stop_motor</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>[Convert if statement to a conditional expression]
-7  void stop_motor(int state)
-       8  {
-       9    (state != 0) ? {
-      10      } : {};
-      11  }</t>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>[Convert integer to Boolean]
+if (state != 0)</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
+          <t>[Use a Boolean variable]
+int state_bool = state != 0;
+if (state_bool)</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
           <t>Fix 1</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>7  void stop_motor(int state)
-       8  {
-       9    (state != 0) ? {
-      10      } : {};
-      11  }</t>
-        </is>
-      </c>
-      <c r="J12" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>if (state != 0)</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>#include &lt;stdint.h&gt;
 void start_motor(void)
@@ -1461,8 +1469,8 @@
 }
 void stop_motor(int state)
 {
-    (state != 0) ? {
-    } : {};
+    if (state != 0)
+    {
     }
 }
 void spin_wait(void)
@@ -1474,24 +1482,24 @@
 }</t>
         </is>
       </c>
-      <c r="L12" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M12" s="10" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N12" s="11" t="inlineStr">
         <is>
           <t>Fix 1 Committed</t>
         </is>
       </c>
-      <c r="N12" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O12" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-07 22:50:20</t>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08 18:06:58</t>
         </is>
       </c>
     </row>
@@ -1504,9 +1512,9 @@
           <t>MISRA-R (Required)</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>14.1</t>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Rule 14.1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1524,70 +1532,116 @@
           <t>spin_wait</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>[Replace atoi with a safer alternative]
-/* Replace atoi with sscanf */
-int i = 0;
-sscanf(some_string, "%d", &amp;i);</t>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>[Correct loop condition]
+8  {
+       9      if (i &gt; 0)
+      10      {
+      11      }
+      12  }
+      13  
+      14  void spin_wait(void)
+      15  {
+      16      int i;
+      17  
+&gt;&gt;&gt;   18      for (i = 10; i &gt; 0; i--)
+      19      {
+      20      }
+      21  }</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Fix 1</t>
+          <t>[Use while loop]
+8  {
+       9      int i = 10;
+      10      while (i &gt; 0)
+      11      {
+      12      }
+      13  }
+      14  
+      15  void spin_wait(void)
+      16  {
+      17      int i;
+      18  
+&gt;&gt;&gt;   19      while (i &gt; 0)
+      20      {
+      21        i--;
+      22      }
+      23  }</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>/* Replace atoi with sscanf */
-int i = 0;
-sscanf(some_string, "%d", &amp;i);</t>
-        </is>
-      </c>
-      <c r="J13" s="13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
-          <t>#include &lt;stdint.h&gt;
+          <t>User Edited</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#include &lt;stdint.h&gt;
 void start_motor(void)
 {
 }
 void stop_motor(int state)
 {
-    if (state)
+    if (i &gt; 0)
     {
     }
 }
 void spin_wait(void)
 {
     int i;
-    sscanf(some_string, "%d", &amp;i);
+    for (i = 10; i &lt; 0; i++)
     {
     }
-}</t>
-        </is>
-      </c>
-      <c r="L13" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M13" s="10" t="inlineStr">
-        <is>
-          <t>Fix 1 Committed</t>
-        </is>
-      </c>
-      <c r="N13" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O13" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-07 22:50:20</t>
+} </t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#include &lt;stdint.h&gt;
+void start_motor(void)
+{
+}
+void stop_motor(int state)
+{
+    if (i &gt; 0)
+    {
+    }
+}
+void spin_wait(void)
+{
+    int i;
+    for (i = 10; i &lt; 0; i++)
+    {
+    }
+} </t>
+        </is>
+      </c>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>User Edited &amp; Committed</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08 18:06:58</t>
         </is>
       </c>
     </row>
@@ -1620,47 +1674,52 @@
           <t>parse_frame</t>
         </is>
       </c>
-      <c r="G14" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I14" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J14" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K14" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L14" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M14" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O14" s="12" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1695,47 +1754,52 @@
           <t>make_mask</t>
         </is>
       </c>
-      <c r="G15" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H15" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I15" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J15" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K15" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L15" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M15" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N15" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O15" s="12" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1770,47 +1834,52 @@
           <t>func</t>
         </is>
       </c>
-      <c r="G16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O16" s="12" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1888,21 +1957,21 @@
           <t>main.c</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>1257, 5124</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Rule 10.3
 Rule 21.6</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>#1257 [Rule 10.3] Narrowing conversion (in main)
 #5124 [Rule 21.6] Standard I/O function used (in main)</t>
@@ -1913,15 +1982,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>#1257: - — -
 #5124: - — -</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-07 22:50:20</t>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08 18:06:58</t>
         </is>
       </c>
     </row>
@@ -1931,15 +2000,15 @@
           <t>utils.c</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>2980, 400, 1460, 1520</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Rule 13.2
 Rule 17.2
@@ -1947,7 +2016,7 @@
 Rule 2.2</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>#2980 [Rule 2.2] Statement has no effect (in helper_add)
 #400 [Rule 13.2] Evaluation order side effects (in update_index)
@@ -1960,7 +2029,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>#2980: - — -
 #400: - — -
@@ -1968,9 +2037,9 @@
 #1520: - — -</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-07 22:50:20</t>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08 18:06:58</t>
         </is>
       </c>
     </row>
@@ -1980,21 +2049,21 @@
           <t>sensor.c</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>2883, 1266</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Rule 10.3
 Rule 9.1</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>#2883 [Rule 9.1] Variable used before initialization (in read_sensor)
 #1266 [Rule 10.3] Narrowing conversion (in scale_value)</t>
@@ -2005,15 +2074,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>#2883: User Edited — User Edited &amp; Committed
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>#2883: - — -
 #1266: - — -</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-07 22:50:20</t>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08 18:06:58</t>
         </is>
       </c>
     </row>
@@ -2023,21 +2092,21 @@
           <t>logger.c</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>3673, 3200</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Rule 17.7
 Rule 8.13</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>#3673 [Rule 8.13] Pointer parameter should be const (in log_message)
 #3200 [Rule 17.7] Return value ignored (in log_message)</t>
@@ -2048,15 +2117,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>#3673: - — -
 #3200: - — -</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-07 22:50:20</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08 18:06:58</t>
         </is>
       </c>
     </row>
@@ -2066,56 +2135,56 @@
           <t>control.c</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>3344, 3340</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>14.1
-14.4</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>#3344 [14.4] Controlling expression not Boolean (in stop_motor)
-#3340 [14.1] Loop never executes (in spin_wait)</t>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Rule 14.1
+Rule 14.4</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>#3344 [Rule 14.4] Controlling expression not Boolean (in stop_motor)
+#3340 [Rule 14.1] Loop never executes (in spin_wait)</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>#include &lt;stdint.h&gt;
+          <t xml:space="preserve">#include &lt;stdint.h&gt;
 void start_motor(void)
 {
 }
 void stop_motor(int state)
 {
-    if (state)
+    if (i &gt; 0)
     {
     }
 }
 void spin_wait(void)
 {
     int i;
-    sscanf(some_string, "%d", &amp;i);
+    for (i = 10; i &lt; 0; i++)
     {
     }
-}</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
+} </t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>#3344: Fix 1 — Fix 1 Committed
-#3340: Fix 1 — Fix 1 Committed</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-07 22:50:20</t>
+#3340: User Edited — User Edited &amp; Committed</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08 18:06:58</t>
         </is>
       </c>
     </row>
@@ -2125,21 +2194,21 @@
           <t>protocol.c</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>1338, 2790</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Rule 12.2
 Rule 17.8</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>#1338 [Rule 17.8] Function parameter modified (in parse_frame)
 #2790 [Rule 12.2] Shift range issue (in make_mask)</t>
@@ -2150,15 +2219,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>#1338: - — -
 #2790: - — -</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-07 22:50:20</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08 18:06:58</t>
         </is>
       </c>
     </row>
@@ -2168,20 +2237,20 @@
           <t>uninit_read.c</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>2883</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Rule 9.1</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>#2883 [Rule 9.1] Variable used before initialization (in func)</t>
         </is>
@@ -2191,14 +2260,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>#2883: - — -</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-07 22:50:20</t>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>2026-04-08 18:06:58</t>
         </is>
       </c>
     </row>

</xml_diff>